<commit_message>
Avancement du 13032026 refonte du modèle + test bentoML
</commit_message>
<xml_diff>
--- a/data_dictionary.xlsx
+++ b/data_dictionary.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tgoth\OneDrive\Bureau\Formation OpenClassRoom\Data Engineer\Projets\6_Anticipez_les_besoins_en_consommation_de_batiments\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E361E04-2AC6-4071-A0A4-403CD8790215}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD4437E9-BE92-429E-A905-C1A4AAB9908D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{03F3F9B1-B293-4043-9854-F162962723C8}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{03F3F9B1-B293-4043-9854-F162962723C8}"/>
   </bookViews>
   <sheets>
     <sheet name="data_dictionary" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="235" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="109">
   <si>
     <t>Colonnes</t>
   </si>
@@ -334,10 +334,25 @@
     <t>yes</t>
   </si>
   <si>
-    <t>À garder pour l'anoalyesse ?</t>
-  </si>
-  <si>
     <t>no</t>
+  </si>
+  <si>
+    <t>À garder pour l'analyse ?</t>
+  </si>
+  <si>
+    <t>Remarques</t>
+  </si>
+  <si>
+    <t>Transformer en nombre d'usage dans le bâtiment</t>
+  </si>
+  <si>
+    <t>target energy</t>
+  </si>
+  <si>
+    <t>target CO2</t>
+  </si>
+  <si>
+    <t>Encoder par la surface moyenne par type</t>
   </si>
 </sst>
 </file>
@@ -427,14 +442,15 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{CDD5762D-AFC2-4714-A10E-6C29C2C659CD}" name="Tableau3" displayName="Tableau3" ref="A1:E47" totalsRowShown="0" headerRowDxfId="1">
-  <autoFilter ref="A1:E47" xr:uid="{CDD5762D-AFC2-4714-A10E-6C29C2C659CD}"/>
-  <tableColumns count="5">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{CDD5762D-AFC2-4714-A10E-6C29C2C659CD}" name="Tableau3" displayName="Tableau3" ref="A1:F47" totalsRowShown="0" headerRowDxfId="1">
+  <autoFilter ref="A1:F47" xr:uid="{CDD5762D-AFC2-4714-A10E-6C29C2C659CD}"/>
+  <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{FCDE9CA3-1643-4A2F-8B51-C4B6402B39EF}" name="Colonnes"/>
     <tableColumn id="2" xr3:uid="{6859DC14-6A4A-4CD8-B313-4F80621C3CAE}" name="Description" dataDxfId="0"/>
     <tableColumn id="3" xr3:uid="{2EF713FA-525D-44CF-A902-70145228FB52}" name="Types"/>
     <tableColumn id="5" xr3:uid="{2B13536E-83AC-4F1D-88C5-CEB948BD3D5A}" name="Variable"/>
-    <tableColumn id="4" xr3:uid="{2FE7F20D-6DF3-487E-B5C7-3182D4234452}" name="À garder pour l'anoalyesse ?"/>
+    <tableColumn id="4" xr3:uid="{2FE7F20D-6DF3-487E-B5C7-3182D4234452}" name="À garder pour l'analyse ?"/>
+    <tableColumn id="6" xr3:uid="{BA4779E4-D2D6-4C5E-9C1A-2CD8E42F1969}" name="Remarques"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -737,7 +753,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8093E335-035B-484E-AA52-9FD90109C23B}">
-  <dimension ref="A1:E47"/>
+  <dimension ref="A1:F47"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="33.140625" bestFit="1" customWidth="1"/>
@@ -745,9 +761,10 @@
     <col min="3" max="3" width="11.5703125" customWidth="1"/>
     <col min="4" max="4" width="14.140625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="27.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="48" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -761,10 +778,13 @@
         <v>98</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+        <v>103</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -778,10 +798,10 @@
         <v>99</v>
       </c>
       <c r="E2" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -795,10 +815,10 @@
         <v>100</v>
       </c>
       <c r="E3" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -815,7 +835,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -829,10 +849,10 @@
         <v>99</v>
       </c>
       <c r="E5" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>11</v>
       </c>
@@ -846,10 +866,10 @@
         <v>99</v>
       </c>
       <c r="E6" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -863,10 +883,10 @@
         <v>99</v>
       </c>
       <c r="E7" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>15</v>
       </c>
@@ -880,10 +900,10 @@
         <v>99</v>
       </c>
       <c r="E8" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>17</v>
       </c>
@@ -897,10 +917,10 @@
         <v>99</v>
       </c>
       <c r="E9" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>19</v>
       </c>
@@ -914,10 +934,10 @@
         <v>99</v>
       </c>
       <c r="E10" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>21</v>
       </c>
@@ -931,10 +951,10 @@
         <v>99</v>
       </c>
       <c r="E11" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>23</v>
       </c>
@@ -948,10 +968,10 @@
         <v>99</v>
       </c>
       <c r="E12" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>25</v>
       </c>
@@ -965,10 +985,10 @@
         <v>99</v>
       </c>
       <c r="E13" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>27</v>
       </c>
@@ -982,10 +1002,10 @@
         <v>99</v>
       </c>
       <c r="E14" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>29</v>
       </c>
@@ -999,10 +1019,10 @@
         <v>99</v>
       </c>
       <c r="E15" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>31</v>
       </c>
@@ -1019,7 +1039,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>33</v>
       </c>
@@ -1036,7 +1056,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>35</v>
       </c>
@@ -1053,7 +1073,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>37</v>
       </c>
@@ -1067,10 +1087,10 @@
         <v>100</v>
       </c>
       <c r="E19" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>39</v>
       </c>
@@ -1084,10 +1104,10 @@
         <v>100</v>
       </c>
       <c r="E20" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>41</v>
       </c>
@@ -1104,7 +1124,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>43</v>
       </c>
@@ -1118,10 +1138,13 @@
         <v>99</v>
       </c>
       <c r="E22" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+        <v>101</v>
+      </c>
+      <c r="F22" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>45</v>
       </c>
@@ -1137,8 +1160,11 @@
       <c r="E23" t="s">
         <v>101</v>
       </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F23" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>47</v>
       </c>
@@ -1152,10 +1178,10 @@
         <v>100</v>
       </c>
       <c r="E24" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>49</v>
       </c>
@@ -1169,10 +1195,10 @@
         <v>99</v>
       </c>
       <c r="E25" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>51</v>
       </c>
@@ -1186,10 +1212,10 @@
         <v>100</v>
       </c>
       <c r="E26" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>53</v>
       </c>
@@ -1203,10 +1229,10 @@
         <v>99</v>
       </c>
       <c r="E27" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>55</v>
       </c>
@@ -1220,10 +1246,10 @@
         <v>100</v>
       </c>
       <c r="E28" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>57</v>
       </c>
@@ -1237,10 +1263,10 @@
         <v>100</v>
       </c>
       <c r="E29" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>59</v>
       </c>
@@ -1257,7 +1283,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>61</v>
       </c>
@@ -1271,10 +1297,10 @@
         <v>100</v>
       </c>
       <c r="E31" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>63</v>
       </c>
@@ -1288,10 +1314,10 @@
         <v>100</v>
       </c>
       <c r="E32" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>65</v>
       </c>
@@ -1305,10 +1331,10 @@
         <v>100</v>
       </c>
       <c r="E33" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>67</v>
       </c>
@@ -1322,10 +1348,10 @@
         <v>100</v>
       </c>
       <c r="E34" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>69</v>
       </c>
@@ -1341,8 +1367,11 @@
       <c r="E35" t="s">
         <v>101</v>
       </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F35" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>71</v>
       </c>
@@ -1356,10 +1385,10 @@
         <v>100</v>
       </c>
       <c r="E36" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>73</v>
       </c>
@@ -1373,10 +1402,10 @@
         <v>100</v>
       </c>
       <c r="E37" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>75</v>
       </c>
@@ -1390,10 +1419,10 @@
         <v>100</v>
       </c>
       <c r="E38" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>77</v>
       </c>
@@ -1407,10 +1436,10 @@
         <v>100</v>
       </c>
       <c r="E39" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>79</v>
       </c>
@@ -1424,10 +1453,10 @@
         <v>100</v>
       </c>
       <c r="E40" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>81</v>
       </c>
@@ -1441,10 +1470,10 @@
         <v>100</v>
       </c>
       <c r="E41" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>83</v>
       </c>
@@ -1458,10 +1487,10 @@
         <v>99</v>
       </c>
       <c r="E42" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>85</v>
       </c>
@@ -1475,10 +1504,10 @@
         <v>99</v>
       </c>
       <c r="E43" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>87</v>
       </c>
@@ -1492,10 +1521,10 @@
         <v>99</v>
       </c>
       <c r="E44" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>89</v>
       </c>
@@ -1509,10 +1538,10 @@
         <v>99</v>
       </c>
       <c r="E45" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>91</v>
       </c>
@@ -1528,8 +1557,11 @@
       <c r="E46" t="s">
         <v>101</v>
       </c>
-    </row>
-    <row r="47" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="F46" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
         <v>93</v>
       </c>
@@ -1543,7 +1575,7 @@
         <v>100</v>
       </c>
       <c r="E47" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Mise à jour dictionnaire des données
</commit_message>
<xml_diff>
--- a/data_dictionary.xlsx
+++ b/data_dictionary.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tgoth\OneDrive\Bureau\Formation OpenClassRoom\Data Engineer\Projets\6_Anticipez_les_besoins_en_consommation_de_batiments\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD4437E9-BE92-429E-A905-C1A4AAB9908D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11164F1D-691D-4DAC-A830-496ECC2C121B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{03F3F9B1-B293-4043-9854-F162962723C8}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{03F3F9B1-B293-4043-9854-F162962723C8}"/>
   </bookViews>
   <sheets>
     <sheet name="data_dictionary" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="101">
   <si>
     <t>Colonnes</t>
   </si>
@@ -329,30 +329,6 @@
   </si>
   <si>
     <t>QUANTITATIVE</t>
-  </si>
-  <si>
-    <t>yes</t>
-  </si>
-  <si>
-    <t>no</t>
-  </si>
-  <si>
-    <t>À garder pour l'analyse ?</t>
-  </si>
-  <si>
-    <t>Remarques</t>
-  </si>
-  <si>
-    <t>Transformer en nombre d'usage dans le bâtiment</t>
-  </si>
-  <si>
-    <t>target energy</t>
-  </si>
-  <si>
-    <t>target CO2</t>
-  </si>
-  <si>
-    <t>Encoder par la surface moyenne par type</t>
   </si>
 </sst>
 </file>
@@ -442,15 +418,13 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{CDD5762D-AFC2-4714-A10E-6C29C2C659CD}" name="Tableau3" displayName="Tableau3" ref="A1:F47" totalsRowShown="0" headerRowDxfId="1">
-  <autoFilter ref="A1:F47" xr:uid="{CDD5762D-AFC2-4714-A10E-6C29C2C659CD}"/>
-  <tableColumns count="6">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{CDD5762D-AFC2-4714-A10E-6C29C2C659CD}" name="Tableau3" displayName="Tableau3" ref="A1:D47" totalsRowShown="0" headerRowDxfId="1">
+  <autoFilter ref="A1:D47" xr:uid="{CDD5762D-AFC2-4714-A10E-6C29C2C659CD}"/>
+  <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{FCDE9CA3-1643-4A2F-8B51-C4B6402B39EF}" name="Colonnes"/>
     <tableColumn id="2" xr3:uid="{6859DC14-6A4A-4CD8-B313-4F80621C3CAE}" name="Description" dataDxfId="0"/>
     <tableColumn id="3" xr3:uid="{2EF713FA-525D-44CF-A902-70145228FB52}" name="Types"/>
     <tableColumn id="5" xr3:uid="{2B13536E-83AC-4F1D-88C5-CEB948BD3D5A}" name="Variable"/>
-    <tableColumn id="4" xr3:uid="{2FE7F20D-6DF3-487E-B5C7-3182D4234452}" name="À garder pour l'analyse ?"/>
-    <tableColumn id="6" xr3:uid="{BA4779E4-D2D6-4C5E-9C1A-2CD8E42F1969}" name="Remarques"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -753,18 +727,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8093E335-035B-484E-AA52-9FD90109C23B}">
-  <dimension ref="A1:F47"/>
+  <dimension ref="A1:D47"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="33.140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="104.7109375" customWidth="1"/>
     <col min="3" max="3" width="11.5703125" customWidth="1"/>
     <col min="4" max="4" width="14.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="27.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="48" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -777,14 +749,8 @@
       <c r="D1" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="E1" s="3" t="s">
-        <v>103</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -797,11 +763,8 @@
       <c r="D2" t="s">
         <v>99</v>
       </c>
-      <c r="E2" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -814,11 +777,8 @@
       <c r="D3" t="s">
         <v>100</v>
       </c>
-      <c r="E3" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -831,11 +791,8 @@
       <c r="D4" t="s">
         <v>99</v>
       </c>
-      <c r="E4" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -848,11 +805,8 @@
       <c r="D5" t="s">
         <v>99</v>
       </c>
-      <c r="E5" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>11</v>
       </c>
@@ -865,11 +819,8 @@
       <c r="D6" t="s">
         <v>99</v>
       </c>
-      <c r="E6" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -882,11 +833,8 @@
       <c r="D7" t="s">
         <v>99</v>
       </c>
-      <c r="E7" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>15</v>
       </c>
@@ -899,11 +847,8 @@
       <c r="D8" t="s">
         <v>99</v>
       </c>
-      <c r="E8" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>17</v>
       </c>
@@ -916,11 +861,8 @@
       <c r="D9" t="s">
         <v>99</v>
       </c>
-      <c r="E9" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>19</v>
       </c>
@@ -933,11 +875,8 @@
       <c r="D10" t="s">
         <v>99</v>
       </c>
-      <c r="E10" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>21</v>
       </c>
@@ -950,11 +889,8 @@
       <c r="D11" t="s">
         <v>99</v>
       </c>
-      <c r="E11" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>23</v>
       </c>
@@ -967,11 +903,8 @@
       <c r="D12" t="s">
         <v>99</v>
       </c>
-      <c r="E12" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>25</v>
       </c>
@@ -984,11 +917,8 @@
       <c r="D13" t="s">
         <v>99</v>
       </c>
-      <c r="E13" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>27</v>
       </c>
@@ -1001,11 +931,8 @@
       <c r="D14" t="s">
         <v>99</v>
       </c>
-      <c r="E14" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>29</v>
       </c>
@@ -1018,11 +945,8 @@
       <c r="D15" t="s">
         <v>99</v>
       </c>
-      <c r="E15" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>31</v>
       </c>
@@ -1035,11 +959,8 @@
       <c r="D16" t="s">
         <v>100</v>
       </c>
-      <c r="E16" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>33</v>
       </c>
@@ -1052,11 +973,8 @@
       <c r="D17" t="s">
         <v>100</v>
       </c>
-      <c r="E17" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>35</v>
       </c>
@@ -1069,11 +987,8 @@
       <c r="D18" t="s">
         <v>100</v>
       </c>
-      <c r="E18" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>37</v>
       </c>
@@ -1086,11 +1001,8 @@
       <c r="D19" t="s">
         <v>100</v>
       </c>
-      <c r="E19" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>39</v>
       </c>
@@ -1103,11 +1015,8 @@
       <c r="D20" t="s">
         <v>100</v>
       </c>
-      <c r="E20" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>41</v>
       </c>
@@ -1120,11 +1029,8 @@
       <c r="D21" t="s">
         <v>100</v>
       </c>
-      <c r="E21" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>43</v>
       </c>
@@ -1137,14 +1043,8 @@
       <c r="D22" t="s">
         <v>99</v>
       </c>
-      <c r="E22" t="s">
-        <v>101</v>
-      </c>
-      <c r="F22" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>45</v>
       </c>
@@ -1157,14 +1057,8 @@
       <c r="D23" t="s">
         <v>99</v>
       </c>
-      <c r="E23" t="s">
-        <v>101</v>
-      </c>
-      <c r="F23" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>47</v>
       </c>
@@ -1177,11 +1071,8 @@
       <c r="D24" t="s">
         <v>100</v>
       </c>
-      <c r="E24" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>49</v>
       </c>
@@ -1194,11 +1085,8 @@
       <c r="D25" t="s">
         <v>99</v>
       </c>
-      <c r="E25" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>51</v>
       </c>
@@ -1211,11 +1099,8 @@
       <c r="D26" t="s">
         <v>100</v>
       </c>
-      <c r="E26" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>53</v>
       </c>
@@ -1228,11 +1113,8 @@
       <c r="D27" t="s">
         <v>99</v>
       </c>
-      <c r="E27" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>55</v>
       </c>
@@ -1245,11 +1127,8 @@
       <c r="D28" t="s">
         <v>100</v>
       </c>
-      <c r="E28" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>57</v>
       </c>
@@ -1262,11 +1141,8 @@
       <c r="D29" t="s">
         <v>100</v>
       </c>
-      <c r="E29" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>59</v>
       </c>
@@ -1279,11 +1155,8 @@
       <c r="D30" t="s">
         <v>100</v>
       </c>
-      <c r="E30" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>61</v>
       </c>
@@ -1296,11 +1169,8 @@
       <c r="D31" t="s">
         <v>100</v>
       </c>
-      <c r="E31" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>63</v>
       </c>
@@ -1313,11 +1183,8 @@
       <c r="D32" t="s">
         <v>100</v>
       </c>
-      <c r="E32" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>65</v>
       </c>
@@ -1330,11 +1197,8 @@
       <c r="D33" t="s">
         <v>100</v>
       </c>
-      <c r="E33" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>67</v>
       </c>
@@ -1347,11 +1211,8 @@
       <c r="D34" t="s">
         <v>100</v>
       </c>
-      <c r="E34" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>69</v>
       </c>
@@ -1364,14 +1225,8 @@
       <c r="D35" t="s">
         <v>100</v>
       </c>
-      <c r="E35" t="s">
-        <v>101</v>
-      </c>
-      <c r="F35" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>71</v>
       </c>
@@ -1384,11 +1239,8 @@
       <c r="D36" t="s">
         <v>100</v>
       </c>
-      <c r="E36" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>73</v>
       </c>
@@ -1401,11 +1253,8 @@
       <c r="D37" t="s">
         <v>100</v>
       </c>
-      <c r="E37" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>75</v>
       </c>
@@ -1418,11 +1267,8 @@
       <c r="D38" t="s">
         <v>100</v>
       </c>
-      <c r="E38" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>77</v>
       </c>
@@ -1435,11 +1281,8 @@
       <c r="D39" t="s">
         <v>100</v>
       </c>
-      <c r="E39" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>79</v>
       </c>
@@ -1452,11 +1295,8 @@
       <c r="D40" t="s">
         <v>100</v>
       </c>
-      <c r="E40" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>81</v>
       </c>
@@ -1469,11 +1309,8 @@
       <c r="D41" t="s">
         <v>100</v>
       </c>
-      <c r="E41" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>83</v>
       </c>
@@ -1486,11 +1323,8 @@
       <c r="D42" t="s">
         <v>99</v>
       </c>
-      <c r="E42" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>85</v>
       </c>
@@ -1503,11 +1337,8 @@
       <c r="D43" t="s">
         <v>99</v>
       </c>
-      <c r="E43" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>87</v>
       </c>
@@ -1520,11 +1351,8 @@
       <c r="D44" t="s">
         <v>99</v>
       </c>
-      <c r="E44" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>89</v>
       </c>
@@ -1537,11 +1365,8 @@
       <c r="D45" t="s">
         <v>99</v>
       </c>
-      <c r="E45" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>91</v>
       </c>
@@ -1554,14 +1379,8 @@
       <c r="D46" t="s">
         <v>100</v>
       </c>
-      <c r="E46" t="s">
-        <v>101</v>
-      </c>
-      <c r="F46" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="47" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    </row>
+    <row r="47" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
         <v>93</v>
       </c>
@@ -1573,9 +1392,6 @@
       </c>
       <c r="D47" s="2" t="s">
         <v>100</v>
-      </c>
-      <c r="E47" s="2" t="s">
-        <v>102</v>
       </c>
     </row>
   </sheetData>

</xml_diff>